<commit_message>
Limit attendance report rows and format totals
</commit_message>
<xml_diff>
--- a/data/list/list_cast.xlsx
+++ b/data/list/list_cast.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\GitHUB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{24DF8679-5FE7-417E-B6E2-1920C47250FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{61103F5A-4058-4E44-9C18-F14C1EDE14B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{9441D692-8DE5-4A5F-83D6-EE7AB38E586A}"/>
+    <workbookView xWindow="4305" yWindow="2460" windowWidth="11175" windowHeight="7785" xr2:uid="{9441D692-8DE5-4A5F-83D6-EE7AB38E586A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t>Sister Luna</t>
     <phoneticPr fontId="1"/>
@@ -114,26 +114,34 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>組　　　／　　　名　　　　／　　　出勤</t>
+    <t>総売上</t>
+    <rPh sb="0" eb="3">
+      <t>ソウウリアゲ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>組</t>
     <rPh sb="0" eb="1">
       <t>クミ</t>
     </rPh>
-    <rPh sb="8" eb="9">
-      <t>メイ</t>
-    </rPh>
-    <rPh sb="17" eb="19">
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>／</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>出勤</t>
+    <rPh sb="0" eb="2">
       <t>シュッキン</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>／　　　　　　　　／　　</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>総売上</t>
-    <rPh sb="0" eb="3">
-      <t>ソウウリアゲ</t>
+    <t>名</t>
+    <rPh sb="0" eb="1">
+      <t>メイ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -657,57 +665,12 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
@@ -724,40 +687,112 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
@@ -770,24 +805,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1131,994 +1148,1002 @@
   </cols>
   <sheetData>
     <row r="1" spans="3:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="I1" s="2"/>
-      <c r="K1" s="1" t="s">
+      <c r="I1" s="1"/>
+      <c r="K1" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="36"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
     </row>
     <row r="2" spans="3:24" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="28"/>
-      <c r="P2" s="28"/>
-      <c r="Q2" s="27" t="s">
+      <c r="K2" s="36"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
+      <c r="N2" s="36"/>
+      <c r="O2" s="37"/>
+      <c r="P2" s="37"/>
+      <c r="Q2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="R2" s="27"/>
-      <c r="S2" s="27" t="s">
+      <c r="R2" s="8"/>
+      <c r="S2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="T2" s="27"/>
-      <c r="U2" s="27" t="s">
+      <c r="T2" s="8"/>
+      <c r="U2" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="V2" s="27" t="s">
+      <c r="V2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="W2" s="27"/>
-      <c r="X2" s="27" t="s">
+      <c r="W2" s="8"/>
+      <c r="X2" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="3:24" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C3" s="17"/>
-      <c r="D3" s="13" t="s">
+      <c r="C3" s="2"/>
+      <c r="D3" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11" t="s">
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11" t="s">
+      <c r="H3" s="18"/>
+      <c r="I3" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11" t="s">
+      <c r="J3" s="18"/>
+      <c r="K3" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11" t="s">
+      <c r="L3" s="18"/>
+      <c r="M3" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11" t="s">
+      <c r="N3" s="18"/>
+      <c r="O3" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="11" t="s">
+      <c r="P3" s="18"/>
+      <c r="Q3" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="R3" s="12"/>
+      <c r="R3" s="19"/>
     </row>
     <row r="4" spans="3:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C4" s="18">
+      <c r="C4" s="3">
         <v>1</v>
       </c>
-      <c r="D4" s="14"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="9"/>
-      <c r="Q4" s="9"/>
-      <c r="R4" s="10"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="21"/>
+      <c r="O4" s="21"/>
+      <c r="P4" s="21"/>
+      <c r="Q4" s="21"/>
+      <c r="R4" s="24"/>
     </row>
     <row r="5" spans="3:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C5" s="19">
+      <c r="C5" s="4">
         <v>2</v>
       </c>
-      <c r="D5" s="15"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="5"/>
-      <c r="R5" s="6"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="23"/>
+      <c r="L5" s="23"/>
+      <c r="M5" s="23"/>
+      <c r="N5" s="23"/>
+      <c r="O5" s="23"/>
+      <c r="P5" s="23"/>
+      <c r="Q5" s="23"/>
+      <c r="R5" s="25"/>
     </row>
     <row r="6" spans="3:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C6" s="19">
+      <c r="C6" s="4">
         <v>3</v>
       </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5"/>
-      <c r="R6" s="6"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="23"/>
+      <c r="N6" s="23"/>
+      <c r="O6" s="23"/>
+      <c r="P6" s="23"/>
+      <c r="Q6" s="23"/>
+      <c r="R6" s="25"/>
     </row>
     <row r="7" spans="3:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C7" s="19">
+      <c r="C7" s="4">
         <v>4</v>
       </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="5"/>
-      <c r="P7" s="5"/>
-      <c r="Q7" s="5"/>
-      <c r="R7" s="6"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="23"/>
+      <c r="P7" s="23"/>
+      <c r="Q7" s="23"/>
+      <c r="R7" s="25"/>
     </row>
     <row r="8" spans="3:24" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C8" s="21">
+      <c r="C8" s="6">
         <v>5</v>
       </c>
-      <c r="D8" s="22"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23"/>
-      <c r="I8" s="23"/>
-      <c r="J8" s="23"/>
-      <c r="K8" s="23"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="23"/>
-      <c r="N8" s="23"/>
-      <c r="O8" s="23"/>
-      <c r="P8" s="23"/>
-      <c r="Q8" s="23"/>
-      <c r="R8" s="24"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="28"/>
+      <c r="K8" s="28"/>
+      <c r="L8" s="28"/>
+      <c r="M8" s="28"/>
+      <c r="N8" s="28"/>
+      <c r="O8" s="28"/>
+      <c r="P8" s="28"/>
+      <c r="Q8" s="28"/>
+      <c r="R8" s="33"/>
     </row>
     <row r="9" spans="3:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C9" s="25">
+      <c r="C9" s="7">
         <v>6</v>
       </c>
-      <c r="D9" s="26"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="3"/>
-      <c r="P9" s="3"/>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="4"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
+      <c r="K9" s="30"/>
+      <c r="L9" s="30"/>
+      <c r="M9" s="30"/>
+      <c r="N9" s="30"/>
+      <c r="O9" s="30"/>
+      <c r="P9" s="30"/>
+      <c r="Q9" s="30"/>
+      <c r="R9" s="34"/>
     </row>
     <row r="10" spans="3:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C10" s="19">
+      <c r="C10" s="4">
         <v>7</v>
       </c>
-      <c r="D10" s="15"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="5"/>
-      <c r="P10" s="5"/>
-      <c r="Q10" s="5"/>
-      <c r="R10" s="6"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="23"/>
+      <c r="O10" s="23"/>
+      <c r="P10" s="23"/>
+      <c r="Q10" s="23"/>
+      <c r="R10" s="25"/>
     </row>
     <row r="11" spans="3:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C11" s="19">
+      <c r="C11" s="4">
         <v>8</v>
       </c>
-      <c r="D11" s="15"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="5"/>
-      <c r="P11" s="5"/>
-      <c r="Q11" s="5"/>
-      <c r="R11" s="6"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="23"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
+      <c r="M11" s="23"/>
+      <c r="N11" s="23"/>
+      <c r="O11" s="23"/>
+      <c r="P11" s="23"/>
+      <c r="Q11" s="23"/>
+      <c r="R11" s="25"/>
     </row>
     <row r="12" spans="3:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C12" s="19">
+      <c r="C12" s="4">
         <v>9</v>
       </c>
-      <c r="D12" s="15"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="5"/>
-      <c r="P12" s="5"/>
-      <c r="Q12" s="5"/>
-      <c r="R12" s="6"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="23"/>
+      <c r="L12" s="23"/>
+      <c r="M12" s="23"/>
+      <c r="N12" s="23"/>
+      <c r="O12" s="23"/>
+      <c r="P12" s="23"/>
+      <c r="Q12" s="23"/>
+      <c r="R12" s="25"/>
     </row>
     <row r="13" spans="3:24" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C13" s="20">
+      <c r="C13" s="5">
         <v>10</v>
       </c>
-      <c r="D13" s="16"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7"/>
-      <c r="M13" s="7"/>
-      <c r="N13" s="7"/>
-      <c r="O13" s="7"/>
-      <c r="P13" s="7"/>
-      <c r="Q13" s="7"/>
-      <c r="R13" s="8"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+      <c r="L13" s="32"/>
+      <c r="M13" s="32"/>
+      <c r="N13" s="32"/>
+      <c r="O13" s="32"/>
+      <c r="P13" s="32"/>
+      <c r="Q13" s="32"/>
+      <c r="R13" s="35"/>
     </row>
     <row r="14" spans="3:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C14" s="18">
+      <c r="C14" s="3">
         <v>11</v>
       </c>
-      <c r="D14" s="14"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-      <c r="M14" s="9"/>
-      <c r="N14" s="9"/>
-      <c r="O14" s="9"/>
-      <c r="P14" s="9"/>
-      <c r="Q14" s="9"/>
-      <c r="R14" s="10"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="21"/>
+      <c r="I14" s="21"/>
+      <c r="J14" s="21"/>
+      <c r="K14" s="21"/>
+      <c r="L14" s="21"/>
+      <c r="M14" s="21"/>
+      <c r="N14" s="21"/>
+      <c r="O14" s="21"/>
+      <c r="P14" s="21"/>
+      <c r="Q14" s="21"/>
+      <c r="R14" s="24"/>
     </row>
     <row r="15" spans="3:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C15" s="19">
+      <c r="C15" s="4">
         <v>12</v>
       </c>
-      <c r="D15" s="15"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-      <c r="O15" s="5"/>
-      <c r="P15" s="5"/>
-      <c r="Q15" s="5"/>
-      <c r="R15" s="6"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="23"/>
+      <c r="J15" s="23"/>
+      <c r="K15" s="23"/>
+      <c r="L15" s="23"/>
+      <c r="M15" s="23"/>
+      <c r="N15" s="23"/>
+      <c r="O15" s="23"/>
+      <c r="P15" s="23"/>
+      <c r="Q15" s="23"/>
+      <c r="R15" s="25"/>
     </row>
     <row r="16" spans="3:24" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C16" s="19">
+      <c r="C16" s="4">
         <v>13</v>
       </c>
-      <c r="D16" s="15"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-      <c r="N16" s="5"/>
-      <c r="O16" s="5"/>
-      <c r="P16" s="5"/>
-      <c r="Q16" s="5"/>
-      <c r="R16" s="6"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="23"/>
+      <c r="M16" s="23"/>
+      <c r="N16" s="23"/>
+      <c r="O16" s="23"/>
+      <c r="P16" s="23"/>
+      <c r="Q16" s="23"/>
+      <c r="R16" s="25"/>
     </row>
     <row r="17" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C17" s="19">
+      <c r="C17" s="4">
         <v>14</v>
       </c>
-      <c r="D17" s="15"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="5"/>
-      <c r="O17" s="5"/>
-      <c r="P17" s="5"/>
-      <c r="Q17" s="5"/>
-      <c r="R17" s="6"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="23"/>
+      <c r="K17" s="23"/>
+      <c r="L17" s="23"/>
+      <c r="M17" s="23"/>
+      <c r="N17" s="23"/>
+      <c r="O17" s="23"/>
+      <c r="P17" s="23"/>
+      <c r="Q17" s="23"/>
+      <c r="R17" s="25"/>
     </row>
     <row r="18" spans="3:18" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C18" s="21">
+      <c r="C18" s="6">
         <v>15</v>
       </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="23"/>
-      <c r="I18" s="23"/>
-      <c r="J18" s="23"/>
-      <c r="K18" s="23"/>
-      <c r="L18" s="23"/>
-      <c r="M18" s="23"/>
-      <c r="N18" s="23"/>
-      <c r="O18" s="23"/>
-      <c r="P18" s="23"/>
-      <c r="Q18" s="23"/>
-      <c r="R18" s="24"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="28"/>
+      <c r="K18" s="28"/>
+      <c r="L18" s="28"/>
+      <c r="M18" s="28"/>
+      <c r="N18" s="28"/>
+      <c r="O18" s="28"/>
+      <c r="P18" s="28"/>
+      <c r="Q18" s="28"/>
+      <c r="R18" s="33"/>
     </row>
     <row r="19" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C19" s="25">
+      <c r="C19" s="7">
         <v>16</v>
       </c>
-      <c r="D19" s="26"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="3"/>
-      <c r="P19" s="3"/>
-      <c r="Q19" s="3"/>
-      <c r="R19" s="4"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="30"/>
+      <c r="J19" s="30"/>
+      <c r="K19" s="30"/>
+      <c r="L19" s="30"/>
+      <c r="M19" s="30"/>
+      <c r="N19" s="30"/>
+      <c r="O19" s="30"/>
+      <c r="P19" s="30"/>
+      <c r="Q19" s="30"/>
+      <c r="R19" s="34"/>
     </row>
     <row r="20" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C20" s="19">
+      <c r="C20" s="4">
         <v>17</v>
       </c>
-      <c r="D20" s="15"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5"/>
-      <c r="P20" s="5"/>
-      <c r="Q20" s="5"/>
-      <c r="R20" s="6"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
+      <c r="J20" s="23"/>
+      <c r="K20" s="23"/>
+      <c r="L20" s="23"/>
+      <c r="M20" s="23"/>
+      <c r="N20" s="23"/>
+      <c r="O20" s="23"/>
+      <c r="P20" s="23"/>
+      <c r="Q20" s="23"/>
+      <c r="R20" s="25"/>
     </row>
     <row r="21" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C21" s="19">
+      <c r="C21" s="4">
         <v>18</v>
       </c>
-      <c r="D21" s="15"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-      <c r="O21" s="5"/>
-      <c r="P21" s="5"/>
-      <c r="Q21" s="5"/>
-      <c r="R21" s="6"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="23"/>
+      <c r="K21" s="23"/>
+      <c r="L21" s="23"/>
+      <c r="M21" s="23"/>
+      <c r="N21" s="23"/>
+      <c r="O21" s="23"/>
+      <c r="P21" s="23"/>
+      <c r="Q21" s="23"/>
+      <c r="R21" s="25"/>
     </row>
     <row r="22" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C22" s="19">
+      <c r="C22" s="4">
         <v>19</v>
       </c>
-      <c r="D22" s="15"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5"/>
-      <c r="M22" s="5"/>
-      <c r="N22" s="5"/>
-      <c r="O22" s="5"/>
-      <c r="P22" s="5"/>
-      <c r="Q22" s="5"/>
-      <c r="R22" s="6"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="23"/>
+      <c r="I22" s="23"/>
+      <c r="J22" s="23"/>
+      <c r="K22" s="23"/>
+      <c r="L22" s="23"/>
+      <c r="M22" s="23"/>
+      <c r="N22" s="23"/>
+      <c r="O22" s="23"/>
+      <c r="P22" s="23"/>
+      <c r="Q22" s="23"/>
+      <c r="R22" s="25"/>
     </row>
     <row r="23" spans="3:18" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C23" s="20">
+      <c r="C23" s="5">
         <v>20</v>
       </c>
-      <c r="D23" s="16"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="7"/>
-      <c r="L23" s="7"/>
-      <c r="M23" s="7"/>
-      <c r="N23" s="7"/>
-      <c r="O23" s="7"/>
-      <c r="P23" s="7"/>
-      <c r="Q23" s="7"/>
-      <c r="R23" s="8"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="32"/>
+      <c r="L23" s="32"/>
+      <c r="M23" s="32"/>
+      <c r="N23" s="32"/>
+      <c r="O23" s="32"/>
+      <c r="P23" s="32"/>
+      <c r="Q23" s="32"/>
+      <c r="R23" s="35"/>
     </row>
     <row r="24" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C24" s="18">
+      <c r="C24" s="3">
         <v>21</v>
       </c>
-      <c r="D24" s="14"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="9"/>
-      <c r="L24" s="9"/>
-      <c r="M24" s="9"/>
-      <c r="N24" s="9"/>
-      <c r="O24" s="9"/>
-      <c r="P24" s="9"/>
-      <c r="Q24" s="9"/>
-      <c r="R24" s="10"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="21"/>
+      <c r="I24" s="21"/>
+      <c r="J24" s="21"/>
+      <c r="K24" s="21"/>
+      <c r="L24" s="21"/>
+      <c r="M24" s="21"/>
+      <c r="N24" s="21"/>
+      <c r="O24" s="21"/>
+      <c r="P24" s="21"/>
+      <c r="Q24" s="21"/>
+      <c r="R24" s="24"/>
     </row>
     <row r="25" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C25" s="19">
+      <c r="C25" s="4">
         <v>22</v>
       </c>
-      <c r="D25" s="15"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
-      <c r="L25" s="5"/>
-      <c r="M25" s="5"/>
-      <c r="N25" s="5"/>
-      <c r="O25" s="5"/>
-      <c r="P25" s="5"/>
-      <c r="Q25" s="5"/>
-      <c r="R25" s="6"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="23"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="23"/>
+      <c r="J25" s="23"/>
+      <c r="K25" s="23"/>
+      <c r="L25" s="23"/>
+      <c r="M25" s="23"/>
+      <c r="N25" s="23"/>
+      <c r="O25" s="23"/>
+      <c r="P25" s="23"/>
+      <c r="Q25" s="23"/>
+      <c r="R25" s="25"/>
     </row>
     <row r="26" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C26" s="19">
+      <c r="C26" s="4">
         <v>23</v>
       </c>
-      <c r="D26" s="15"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
-      <c r="L26" s="5"/>
-      <c r="M26" s="5"/>
-      <c r="N26" s="5"/>
-      <c r="O26" s="5"/>
-      <c r="P26" s="5"/>
-      <c r="Q26" s="5"/>
-      <c r="R26" s="6"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="23"/>
+      <c r="H26" s="23"/>
+      <c r="I26" s="23"/>
+      <c r="J26" s="23"/>
+      <c r="K26" s="23"/>
+      <c r="L26" s="23"/>
+      <c r="M26" s="23"/>
+      <c r="N26" s="23"/>
+      <c r="O26" s="23"/>
+      <c r="P26" s="23"/>
+      <c r="Q26" s="23"/>
+      <c r="R26" s="25"/>
     </row>
     <row r="27" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C27" s="19">
+      <c r="C27" s="4">
         <v>24</v>
       </c>
-      <c r="D27" s="15"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
-      <c r="L27" s="5"/>
-      <c r="M27" s="5"/>
-      <c r="N27" s="5"/>
-      <c r="O27" s="5"/>
-      <c r="P27" s="5"/>
-      <c r="Q27" s="5"/>
-      <c r="R27" s="6"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="23"/>
+      <c r="H27" s="23"/>
+      <c r="I27" s="23"/>
+      <c r="J27" s="23"/>
+      <c r="K27" s="23"/>
+      <c r="L27" s="23"/>
+      <c r="M27" s="23"/>
+      <c r="N27" s="23"/>
+      <c r="O27" s="23"/>
+      <c r="P27" s="23"/>
+      <c r="Q27" s="23"/>
+      <c r="R27" s="25"/>
     </row>
     <row r="28" spans="3:18" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C28" s="21">
+      <c r="C28" s="6">
         <v>25</v>
       </c>
-      <c r="D28" s="22"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="23"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="23"/>
-      <c r="K28" s="23"/>
-      <c r="L28" s="23"/>
-      <c r="M28" s="23"/>
-      <c r="N28" s="23"/>
-      <c r="O28" s="23"/>
-      <c r="P28" s="23"/>
-      <c r="Q28" s="23"/>
-      <c r="R28" s="24"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="28"/>
+      <c r="I28" s="28"/>
+      <c r="J28" s="28"/>
+      <c r="K28" s="28"/>
+      <c r="L28" s="28"/>
+      <c r="M28" s="28"/>
+      <c r="N28" s="28"/>
+      <c r="O28" s="28"/>
+      <c r="P28" s="28"/>
+      <c r="Q28" s="28"/>
+      <c r="R28" s="33"/>
     </row>
     <row r="29" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C29" s="25">
+      <c r="C29" s="7">
         <v>26</v>
       </c>
-      <c r="D29" s="26"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
-      <c r="G29" s="3"/>
-      <c r="H29" s="3"/>
-      <c r="I29" s="3"/>
-      <c r="J29" s="3"/>
-      <c r="K29" s="3"/>
-      <c r="L29" s="3"/>
-      <c r="M29" s="3"/>
-      <c r="N29" s="3"/>
-      <c r="O29" s="3"/>
-      <c r="P29" s="3"/>
-      <c r="Q29" s="3"/>
-      <c r="R29" s="4"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="30"/>
+      <c r="J29" s="30"/>
+      <c r="K29" s="30"/>
+      <c r="L29" s="30"/>
+      <c r="M29" s="30"/>
+      <c r="N29" s="30"/>
+      <c r="O29" s="30"/>
+      <c r="P29" s="30"/>
+      <c r="Q29" s="30"/>
+      <c r="R29" s="34"/>
     </row>
     <row r="30" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C30" s="19">
+      <c r="C30" s="4">
         <v>27</v>
       </c>
-      <c r="D30" s="15"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
-      <c r="J30" s="5"/>
-      <c r="K30" s="5"/>
-      <c r="L30" s="5"/>
-      <c r="M30" s="5"/>
-      <c r="N30" s="5"/>
-      <c r="O30" s="5"/>
-      <c r="P30" s="5"/>
-      <c r="Q30" s="5"/>
-      <c r="R30" s="6"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="23"/>
+      <c r="I30" s="23"/>
+      <c r="J30" s="23"/>
+      <c r="K30" s="23"/>
+      <c r="L30" s="23"/>
+      <c r="M30" s="23"/>
+      <c r="N30" s="23"/>
+      <c r="O30" s="23"/>
+      <c r="P30" s="23"/>
+      <c r="Q30" s="23"/>
+      <c r="R30" s="25"/>
     </row>
     <row r="31" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C31" s="19">
+      <c r="C31" s="4">
         <v>28</v>
       </c>
-      <c r="D31" s="15"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="5"/>
-      <c r="J31" s="5"/>
-      <c r="K31" s="5"/>
-      <c r="L31" s="5"/>
-      <c r="M31" s="5"/>
-      <c r="N31" s="5"/>
-      <c r="O31" s="5"/>
-      <c r="P31" s="5"/>
-      <c r="Q31" s="5"/>
-      <c r="R31" s="6"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="23"/>
+      <c r="H31" s="23"/>
+      <c r="I31" s="23"/>
+      <c r="J31" s="23"/>
+      <c r="K31" s="23"/>
+      <c r="L31" s="23"/>
+      <c r="M31" s="23"/>
+      <c r="N31" s="23"/>
+      <c r="O31" s="23"/>
+      <c r="P31" s="23"/>
+      <c r="Q31" s="23"/>
+      <c r="R31" s="25"/>
     </row>
     <row r="32" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C32" s="19">
+      <c r="C32" s="4">
         <v>29</v>
       </c>
-      <c r="D32" s="15"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="5"/>
-      <c r="J32" s="5"/>
-      <c r="K32" s="5"/>
-      <c r="L32" s="5"/>
-      <c r="M32" s="5"/>
-      <c r="N32" s="5"/>
-      <c r="O32" s="5"/>
-      <c r="P32" s="5"/>
-      <c r="Q32" s="5"/>
-      <c r="R32" s="6"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
+      <c r="G32" s="23"/>
+      <c r="H32" s="23"/>
+      <c r="I32" s="23"/>
+      <c r="J32" s="23"/>
+      <c r="K32" s="23"/>
+      <c r="L32" s="23"/>
+      <c r="M32" s="23"/>
+      <c r="N32" s="23"/>
+      <c r="O32" s="23"/>
+      <c r="P32" s="23"/>
+      <c r="Q32" s="23"/>
+      <c r="R32" s="25"/>
     </row>
     <row r="33" spans="3:18" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C33" s="20">
+      <c r="C33" s="5">
         <v>30</v>
       </c>
-      <c r="D33" s="16"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="7"/>
-      <c r="J33" s="7"/>
-      <c r="K33" s="7"/>
-      <c r="L33" s="7"/>
-      <c r="M33" s="7"/>
-      <c r="N33" s="7"/>
-      <c r="O33" s="7"/>
-      <c r="P33" s="7"/>
-      <c r="Q33" s="7"/>
-      <c r="R33" s="8"/>
+      <c r="D33" s="31"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="32"/>
+      <c r="J33" s="32"/>
+      <c r="K33" s="32"/>
+      <c r="L33" s="32"/>
+      <c r="M33" s="32"/>
+      <c r="N33" s="32"/>
+      <c r="O33" s="32"/>
+      <c r="P33" s="32"/>
+      <c r="Q33" s="32"/>
+      <c r="R33" s="35"/>
     </row>
     <row r="34" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C34" s="18">
+      <c r="C34" s="3">
         <v>31</v>
       </c>
-      <c r="D34" s="14"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="9"/>
-      <c r="H34" s="9"/>
-      <c r="I34" s="9"/>
-      <c r="J34" s="9"/>
-      <c r="K34" s="9"/>
-      <c r="L34" s="9"/>
-      <c r="M34" s="9"/>
-      <c r="N34" s="9"/>
-      <c r="O34" s="9"/>
-      <c r="P34" s="9"/>
-      <c r="Q34" s="9"/>
-      <c r="R34" s="10"/>
+      <c r="D34" s="20"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="21"/>
+      <c r="G34" s="21"/>
+      <c r="H34" s="21"/>
+      <c r="I34" s="21"/>
+      <c r="J34" s="21"/>
+      <c r="K34" s="21"/>
+      <c r="L34" s="21"/>
+      <c r="M34" s="21"/>
+      <c r="N34" s="21"/>
+      <c r="O34" s="21"/>
+      <c r="P34" s="21"/>
+      <c r="Q34" s="21"/>
+      <c r="R34" s="24"/>
     </row>
     <row r="35" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C35" s="19">
+      <c r="C35" s="4">
         <v>32</v>
       </c>
-      <c r="D35" s="15"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="5"/>
-      <c r="J35" s="5"/>
-      <c r="K35" s="5"/>
-      <c r="L35" s="5"/>
-      <c r="M35" s="5"/>
-      <c r="N35" s="5"/>
-      <c r="O35" s="5"/>
-      <c r="P35" s="5"/>
-      <c r="Q35" s="5"/>
-      <c r="R35" s="6"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="23"/>
+      <c r="F35" s="23"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="23"/>
+      <c r="I35" s="23"/>
+      <c r="J35" s="23"/>
+      <c r="K35" s="23"/>
+      <c r="L35" s="23"/>
+      <c r="M35" s="23"/>
+      <c r="N35" s="23"/>
+      <c r="O35" s="23"/>
+      <c r="P35" s="23"/>
+      <c r="Q35" s="23"/>
+      <c r="R35" s="25"/>
     </row>
     <row r="36" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C36" s="19">
+      <c r="C36" s="4">
         <v>33</v>
       </c>
-      <c r="D36" s="15"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5"/>
-      <c r="J36" s="5"/>
-      <c r="K36" s="5"/>
-      <c r="L36" s="5"/>
-      <c r="M36" s="5"/>
-      <c r="N36" s="5"/>
-      <c r="O36" s="5"/>
-      <c r="P36" s="5"/>
-      <c r="Q36" s="5"/>
-      <c r="R36" s="6"/>
+      <c r="D36" s="22"/>
+      <c r="E36" s="23"/>
+      <c r="F36" s="23"/>
+      <c r="G36" s="23"/>
+      <c r="H36" s="23"/>
+      <c r="I36" s="23"/>
+      <c r="J36" s="23"/>
+      <c r="K36" s="23"/>
+      <c r="L36" s="23"/>
+      <c r="M36" s="23"/>
+      <c r="N36" s="23"/>
+      <c r="O36" s="23"/>
+      <c r="P36" s="23"/>
+      <c r="Q36" s="23"/>
+      <c r="R36" s="25"/>
     </row>
     <row r="37" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C37" s="19">
+      <c r="C37" s="4">
         <v>34</v>
       </c>
-      <c r="D37" s="15"/>
-      <c r="E37" s="5"/>
-      <c r="F37" s="5"/>
-      <c r="G37" s="5"/>
-      <c r="H37" s="5"/>
-      <c r="I37" s="5"/>
-      <c r="J37" s="5"/>
-      <c r="K37" s="5"/>
-      <c r="L37" s="5"/>
-      <c r="M37" s="5"/>
-      <c r="N37" s="5"/>
-      <c r="O37" s="5"/>
-      <c r="P37" s="5"/>
-      <c r="Q37" s="5"/>
-      <c r="R37" s="6"/>
+      <c r="D37" s="22"/>
+      <c r="E37" s="23"/>
+      <c r="F37" s="23"/>
+      <c r="G37" s="23"/>
+      <c r="H37" s="23"/>
+      <c r="I37" s="23"/>
+      <c r="J37" s="23"/>
+      <c r="K37" s="23"/>
+      <c r="L37" s="23"/>
+      <c r="M37" s="23"/>
+      <c r="N37" s="23"/>
+      <c r="O37" s="23"/>
+      <c r="P37" s="23"/>
+      <c r="Q37" s="23"/>
+      <c r="R37" s="25"/>
     </row>
     <row r="38" spans="3:18" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C38" s="20">
+      <c r="C38" s="5">
         <v>35</v>
       </c>
-      <c r="D38" s="16"/>
-      <c r="E38" s="7"/>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
-      <c r="H38" s="7"/>
-      <c r="I38" s="7"/>
-      <c r="J38" s="7"/>
-      <c r="K38" s="7"/>
-      <c r="L38" s="7"/>
-      <c r="M38" s="7"/>
-      <c r="N38" s="7"/>
-      <c r="O38" s="7"/>
-      <c r="P38" s="7"/>
-      <c r="Q38" s="7"/>
-      <c r="R38" s="8"/>
+      <c r="D38" s="31"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="32"/>
+      <c r="J38" s="32"/>
+      <c r="K38" s="32"/>
+      <c r="L38" s="32"/>
+      <c r="M38" s="32"/>
+      <c r="N38" s="32"/>
+      <c r="O38" s="32"/>
+      <c r="P38" s="32"/>
+      <c r="Q38" s="32"/>
+      <c r="R38" s="35"/>
     </row>
     <row r="39" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C39" s="18">
+      <c r="C39" s="3">
         <v>36</v>
       </c>
-      <c r="D39" s="14"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="9"/>
-      <c r="G39" s="9"/>
-      <c r="H39" s="9"/>
-      <c r="I39" s="9"/>
-      <c r="J39" s="9"/>
-      <c r="K39" s="9"/>
-      <c r="L39" s="9"/>
-      <c r="M39" s="9"/>
-      <c r="N39" s="9"/>
-      <c r="O39" s="9"/>
-      <c r="P39" s="9"/>
-      <c r="Q39" s="9"/>
-      <c r="R39" s="10"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="21"/>
+      <c r="F39" s="21"/>
+      <c r="G39" s="21"/>
+      <c r="H39" s="21"/>
+      <c r="I39" s="21"/>
+      <c r="J39" s="21"/>
+      <c r="K39" s="21"/>
+      <c r="L39" s="21"/>
+      <c r="M39" s="21"/>
+      <c r="N39" s="21"/>
+      <c r="O39" s="21"/>
+      <c r="P39" s="21"/>
+      <c r="Q39" s="21"/>
+      <c r="R39" s="24"/>
     </row>
     <row r="40" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C40" s="19">
+      <c r="C40" s="4">
         <v>37</v>
       </c>
-      <c r="D40" s="15"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-      <c r="I40" s="5"/>
-      <c r="J40" s="5"/>
-      <c r="K40" s="5"/>
-      <c r="L40" s="5"/>
-      <c r="M40" s="5"/>
-      <c r="N40" s="5"/>
-      <c r="O40" s="5"/>
-      <c r="P40" s="5"/>
-      <c r="Q40" s="5"/>
-      <c r="R40" s="6"/>
+      <c r="D40" s="22"/>
+      <c r="E40" s="23"/>
+      <c r="F40" s="23"/>
+      <c r="G40" s="23"/>
+      <c r="H40" s="23"/>
+      <c r="I40" s="23"/>
+      <c r="J40" s="23"/>
+      <c r="K40" s="23"/>
+      <c r="L40" s="23"/>
+      <c r="M40" s="23"/>
+      <c r="N40" s="23"/>
+      <c r="O40" s="23"/>
+      <c r="P40" s="23"/>
+      <c r="Q40" s="23"/>
+      <c r="R40" s="25"/>
     </row>
     <row r="41" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C41" s="19">
+      <c r="C41" s="4">
         <v>38</v>
       </c>
-      <c r="D41" s="15"/>
-      <c r="E41" s="5"/>
-      <c r="F41" s="5"/>
-      <c r="G41" s="5"/>
-      <c r="H41" s="5"/>
-      <c r="I41" s="5"/>
-      <c r="J41" s="5"/>
-      <c r="K41" s="5"/>
-      <c r="L41" s="5"/>
-      <c r="M41" s="5"/>
-      <c r="N41" s="5"/>
-      <c r="O41" s="5"/>
-      <c r="P41" s="5"/>
-      <c r="Q41" s="5"/>
-      <c r="R41" s="6"/>
+      <c r="D41" s="22"/>
+      <c r="E41" s="23"/>
+      <c r="F41" s="23"/>
+      <c r="G41" s="23"/>
+      <c r="H41" s="23"/>
+      <c r="I41" s="23"/>
+      <c r="J41" s="23"/>
+      <c r="K41" s="23"/>
+      <c r="L41" s="23"/>
+      <c r="M41" s="23"/>
+      <c r="N41" s="23"/>
+      <c r="O41" s="23"/>
+      <c r="P41" s="23"/>
+      <c r="Q41" s="23"/>
+      <c r="R41" s="25"/>
     </row>
     <row r="42" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C42" s="19">
+      <c r="C42" s="4">
         <v>39</v>
       </c>
-      <c r="D42" s="15"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
-      <c r="G42" s="5"/>
-      <c r="H42" s="5"/>
-      <c r="I42" s="5"/>
-      <c r="J42" s="5"/>
-      <c r="K42" s="5"/>
-      <c r="L42" s="5"/>
-      <c r="M42" s="5"/>
-      <c r="N42" s="5"/>
-      <c r="O42" s="5"/>
-      <c r="P42" s="5"/>
-      <c r="Q42" s="5"/>
-      <c r="R42" s="6"/>
+      <c r="D42" s="22"/>
+      <c r="E42" s="23"/>
+      <c r="F42" s="23"/>
+      <c r="G42" s="23"/>
+      <c r="H42" s="23"/>
+      <c r="I42" s="23"/>
+      <c r="J42" s="23"/>
+      <c r="K42" s="23"/>
+      <c r="L42" s="23"/>
+      <c r="M42" s="23"/>
+      <c r="N42" s="23"/>
+      <c r="O42" s="23"/>
+      <c r="P42" s="23"/>
+      <c r="Q42" s="23"/>
+      <c r="R42" s="25"/>
     </row>
     <row r="43" spans="3:18" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C43" s="20">
+      <c r="C43" s="5">
         <v>40</v>
       </c>
-      <c r="D43" s="16"/>
-      <c r="E43" s="7"/>
-      <c r="F43" s="7"/>
-      <c r="G43" s="7"/>
-      <c r="H43" s="7"/>
-      <c r="I43" s="7"/>
-      <c r="J43" s="7"/>
-      <c r="K43" s="7"/>
-      <c r="L43" s="7"/>
-      <c r="M43" s="7"/>
-      <c r="N43" s="7"/>
-      <c r="O43" s="7"/>
-      <c r="P43" s="7"/>
-      <c r="Q43" s="7"/>
-      <c r="R43" s="8"/>
+      <c r="D43" s="31"/>
+      <c r="E43" s="32"/>
+      <c r="F43" s="32"/>
+      <c r="G43" s="32"/>
+      <c r="H43" s="32"/>
+      <c r="I43" s="32"/>
+      <c r="J43" s="32"/>
+      <c r="K43" s="32"/>
+      <c r="L43" s="32"/>
+      <c r="M43" s="32"/>
+      <c r="N43" s="32"/>
+      <c r="O43" s="32"/>
+      <c r="P43" s="32"/>
+      <c r="Q43" s="32"/>
+      <c r="R43" s="35"/>
     </row>
     <row r="44" spans="3:18" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C44" s="29" t="s">
+      <c r="C44" s="9"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H44" s="10"/>
+      <c r="I44" s="10"/>
+      <c r="J44" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="K44" s="10"/>
+      <c r="L44" s="10"/>
+      <c r="M44" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="N44" s="10"/>
+      <c r="O44" s="10"/>
+      <c r="P44" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q44" s="10"/>
+      <c r="R44" s="11"/>
+    </row>
+    <row r="45" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C45" s="14"/>
+      <c r="D45" s="12"/>
+      <c r="E45" s="12"/>
+      <c r="F45" s="12"/>
+      <c r="G45" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="H45" s="12"/>
+      <c r="I45" s="12"/>
+      <c r="J45" s="12"/>
+      <c r="K45" s="12"/>
+      <c r="L45" s="12"/>
+      <c r="M45" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="N45" s="12"/>
+      <c r="O45" s="12"/>
+      <c r="P45" s="12"/>
+      <c r="Q45" s="12"/>
+      <c r="R45" s="16"/>
+    </row>
+    <row r="46" spans="3:18" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="C46" s="15"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="13"/>
+      <c r="F46" s="13"/>
+      <c r="G46" s="13"/>
+      <c r="H46" s="13"/>
+      <c r="I46" s="13"/>
+      <c r="J46" s="13"/>
+      <c r="K46" s="13"/>
+      <c r="L46" s="13"/>
+      <c r="M46" s="13"/>
+      <c r="N46" s="13"/>
+      <c r="O46" s="13"/>
+      <c r="P46" s="13"/>
+      <c r="Q46" s="13"/>
+      <c r="R46" s="17"/>
+    </row>
+    <row r="47" spans="3:18" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="C47" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="D44" s="30"/>
-      <c r="E44" s="30"/>
-      <c r="F44" s="30"/>
-      <c r="G44" s="30"/>
-      <c r="H44" s="30"/>
-      <c r="I44" s="30"/>
-      <c r="J44" s="30"/>
-      <c r="K44" s="30"/>
-      <c r="L44" s="30"/>
-      <c r="M44" s="30"/>
-      <c r="N44" s="30"/>
-      <c r="O44" s="30"/>
-      <c r="P44" s="30"/>
-      <c r="Q44" s="30"/>
-      <c r="R44" s="31"/>
-    </row>
-    <row r="45" spans="3:18" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C45" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="D45" s="39"/>
-      <c r="E45" s="39"/>
-      <c r="F45" s="39"/>
-      <c r="G45" s="39"/>
-      <c r="H45" s="39"/>
-      <c r="I45" s="39"/>
-      <c r="J45" s="39"/>
-      <c r="K45" s="39"/>
-      <c r="L45" s="39"/>
-      <c r="M45" s="39"/>
-      <c r="N45" s="39"/>
-      <c r="O45" s="39"/>
-      <c r="P45" s="39"/>
-      <c r="Q45" s="39"/>
-      <c r="R45" s="40"/>
-    </row>
-    <row r="46" spans="3:18" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C46" s="38"/>
-      <c r="D46" s="39"/>
-      <c r="E46" s="39"/>
-      <c r="F46" s="39"/>
-      <c r="G46" s="39"/>
-      <c r="H46" s="39"/>
-      <c r="I46" s="39"/>
-      <c r="J46" s="39"/>
-      <c r="K46" s="39"/>
-      <c r="L46" s="39"/>
-      <c r="M46" s="39"/>
-      <c r="N46" s="39"/>
-      <c r="O46" s="39"/>
-      <c r="P46" s="39"/>
-      <c r="Q46" s="39"/>
-      <c r="R46" s="40"/>
-    </row>
-    <row r="47" spans="3:18" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C47" s="41" t="s">
-        <v>15</v>
-      </c>
-      <c r="D47" s="42"/>
-      <c r="E47" s="42"/>
-      <c r="F47" s="42"/>
-      <c r="G47" s="42"/>
-      <c r="H47" s="42"/>
-      <c r="I47" s="42"/>
-      <c r="J47" s="42"/>
-      <c r="K47" s="42"/>
-      <c r="L47" s="42"/>
-      <c r="M47" s="42"/>
-      <c r="N47" s="42"/>
-      <c r="O47" s="42"/>
-      <c r="P47" s="42"/>
-      <c r="Q47" s="42"/>
-      <c r="R47" s="43"/>
+      <c r="D47" s="39"/>
+      <c r="E47" s="39"/>
+      <c r="F47" s="39"/>
+      <c r="G47" s="39"/>
+      <c r="H47" s="39"/>
+      <c r="I47" s="39"/>
+      <c r="J47" s="39"/>
+      <c r="K47" s="39"/>
+      <c r="L47" s="39"/>
+      <c r="M47" s="39"/>
+      <c r="N47" s="39"/>
+      <c r="O47" s="39"/>
+      <c r="P47" s="39"/>
+      <c r="Q47" s="39"/>
+      <c r="R47" s="40"/>
     </row>
     <row r="48" spans="3:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="C48" s="32"/>
-      <c r="D48" s="33"/>
-      <c r="E48" s="33"/>
-      <c r="F48" s="33"/>
-      <c r="G48" s="33"/>
-      <c r="H48" s="33"/>
-      <c r="I48" s="33"/>
-      <c r="J48" s="33"/>
-      <c r="K48" s="33"/>
-      <c r="L48" s="33"/>
-      <c r="M48" s="33"/>
-      <c r="N48" s="33"/>
-      <c r="O48" s="33"/>
-      <c r="P48" s="33"/>
-      <c r="Q48" s="33"/>
-      <c r="R48" s="34"/>
+      <c r="C48" s="41"/>
+      <c r="D48" s="42"/>
+      <c r="E48" s="42"/>
+      <c r="F48" s="42"/>
+      <c r="G48" s="42"/>
+      <c r="H48" s="42"/>
+      <c r="I48" s="42"/>
+      <c r="J48" s="42"/>
+      <c r="K48" s="42"/>
+      <c r="L48" s="42"/>
+      <c r="M48" s="42"/>
+      <c r="N48" s="42"/>
+      <c r="O48" s="42"/>
+      <c r="P48" s="42"/>
+      <c r="Q48" s="42"/>
+      <c r="R48" s="43"/>
     </row>
     <row r="49" spans="3:18" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="C49" s="35"/>
-      <c r="D49" s="36"/>
-      <c r="E49" s="36"/>
-      <c r="F49" s="36"/>
-      <c r="G49" s="36"/>
-      <c r="H49" s="36"/>
-      <c r="I49" s="36"/>
-      <c r="J49" s="36"/>
-      <c r="K49" s="36"/>
-      <c r="L49" s="36"/>
-      <c r="M49" s="36"/>
-      <c r="N49" s="36"/>
-      <c r="O49" s="36"/>
-      <c r="P49" s="36"/>
-      <c r="Q49" s="36"/>
-      <c r="R49" s="37"/>
+      <c r="C49" s="44"/>
+      <c r="D49" s="45"/>
+      <c r="E49" s="45"/>
+      <c r="F49" s="45"/>
+      <c r="G49" s="45"/>
+      <c r="H49" s="45"/>
+      <c r="I49" s="45"/>
+      <c r="J49" s="45"/>
+      <c r="K49" s="45"/>
+      <c r="L49" s="45"/>
+      <c r="M49" s="45"/>
+      <c r="N49" s="45"/>
+      <c r="O49" s="45"/>
+      <c r="P49" s="45"/>
+      <c r="Q49" s="45"/>
+      <c r="R49" s="46"/>
     </row>
   </sheetData>
-  <mergeCells count="293">
+  <mergeCells count="296">
     <mergeCell ref="K1:N2"/>
     <mergeCell ref="O2:P2"/>
-    <mergeCell ref="C44:R44"/>
-    <mergeCell ref="C45:R46"/>
     <mergeCell ref="C47:R47"/>
     <mergeCell ref="C48:R49"/>
     <mergeCell ref="G43:H43"/>
@@ -2365,22 +2390,10 @@
     <mergeCell ref="D33:F33"/>
     <mergeCell ref="D34:F34"/>
     <mergeCell ref="D35:F35"/>
-    <mergeCell ref="O4:P4"/>
-    <mergeCell ref="O5:P5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="D29:F29"/>
-    <mergeCell ref="D30:F30"/>
     <mergeCell ref="D31:F31"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D13:F13"/>
     <mergeCell ref="D14:F14"/>
     <mergeCell ref="D15:F15"/>
     <mergeCell ref="D16:F16"/>
@@ -2390,9 +2403,22 @@
     <mergeCell ref="D8:F8"/>
     <mergeCell ref="D9:F9"/>
     <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="D30:F30"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="G45:G46"/>
+    <mergeCell ref="M45:M46"/>
+    <mergeCell ref="C45:F46"/>
+    <mergeCell ref="H45:L46"/>
+    <mergeCell ref="N45:R46"/>
     <mergeCell ref="O3:P3"/>
     <mergeCell ref="Q3:R3"/>
     <mergeCell ref="D4:F4"/>
@@ -2408,6 +2434,10 @@
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="K3:L3"/>
     <mergeCell ref="M3:N3"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="O5:P5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="I6:J6"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>